<commit_message>
refactor(tests): regenerate fixtures + template after dropping pricing/stock
- Updates fixture generators to 7-column TEMPLATE_COLUMNS
- Regenerates good/with-errors/header-mismatch .xlsx
- Regenerates public/templates/catalog-import-template.xlsx
- Drops "Open value" assertion from dashboard.spec.ts
- Replaces "bad_type" assertion with "duplicate_in_file" in catalog-import.spec.ts

Note: tests/fixtures/catalog-import/big.xlsx is gitignored; regenerated locally
via generate-big.ts and not committed.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/catalog-import-template.xlsx
+++ b/public/templates/catalog-import-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>sku</t>
   </si>
@@ -25,15 +25,6 @@
     <t>unit</t>
   </si>
   <si>
-    <t>unit_price</t>
-  </si>
-  <si>
-    <t>on_hand</t>
-  </si>
-  <si>
-    <t>stock_state</t>
-  </si>
-  <si>
     <t>vendor_code</t>
   </si>
   <si>
@@ -55,9 +46,6 @@
     <t>pcs</t>
   </si>
   <si>
-    <t>in-stock</t>
-  </si>
-  <si>
     <t>MSR</t>
   </si>
   <si>
@@ -86,9 +74,6 @@
   </si>
   <si>
     <t>ST</t>
-  </si>
-  <si>
-    <t>low-stock</t>
   </si>
   <si>
     <t>DK</t>
@@ -478,21 +463,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="10" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="7" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -514,110 +496,74 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2">
-        <v>0.012</v>
-      </c>
-      <c r="F2">
-        <v>100</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="G3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>18</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3">
-        <v>0.018</v>
-      </c>
-      <c r="F3">
-        <v>80</v>
-      </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="F4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" t="s">
+      <c r="G4" t="s">
         <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4">
-        <v>1.85</v>
-      </c>
-      <c r="F4">
-        <v>20</v>
-      </c>
-      <c r="G4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>